<commit_message>
progress: 7 village workbooks (sivaramans-llin 2026-10-08T18:05:26Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Chennavaram_13.464802_80.149579.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Chennavaram_13.464802_80.149579.xlsx
@@ -1418,6 +1418,11 @@
           <t>173</t>
         </is>
       </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1425,6 +1430,11 @@
           <t>174</t>
         </is>
       </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1432,6 +1442,11 @@
           <t>175</t>
         </is>
       </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1439,6 +1454,11 @@
           <t>176</t>
         </is>
       </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1446,6 +1466,11 @@
           <t>177</t>
         </is>
       </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1453,6 +1478,11 @@
           <t>178</t>
         </is>
       </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -1460,6 +1490,11 @@
           <t>179</t>
         </is>
       </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -1467,6 +1502,11 @@
           <t>18</t>
         </is>
       </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 2A, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -1474,6 +1514,11 @@
           <t>180</t>
         </is>
       </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1481,6 +1526,11 @@
           <t>181</t>
         </is>
       </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -1488,6 +1538,11 @@
           <t>182</t>
         </is>
       </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -1495,6 +1550,11 @@
           <t>183</t>
         </is>
       </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C1, 2C2, 3A, 3B, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -1502,6 +1562,11 @@
           <t>184</t>
         </is>
       </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -1509,6 +1574,11 @@
           <t>185</t>
         </is>
       </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -1516,6 +1586,11 @@
           <t>186</t>
         </is>
       </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -1523,6 +1598,11 @@
           <t>187</t>
         </is>
       </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -1530,6 +1610,11 @@
           <t>188</t>
         </is>
       </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -1537,6 +1622,11 @@
           <t>189</t>
         </is>
       </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B, 1C, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -1544,6 +1634,11 @@
           <t>19</t>
         </is>
       </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -1551,6 +1646,11 @@
           <t>190</t>
         </is>
       </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -1558,6 +1658,11 @@
           <t>191</t>
         </is>
       </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -1565,6 +1670,11 @@
           <t>192</t>
         </is>
       </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -1572,6 +1682,11 @@
           <t>193</t>
         </is>
       </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 3A, 3B, 3C, 3D, 4, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -1579,6 +1694,11 @@
           <t>194</t>
         </is>
       </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -1586,6 +1706,11 @@
           <t>195</t>
         </is>
       </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C, 3D, 3E</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -1593,6 +1718,11 @@
           <t>196</t>
         </is>
       </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4A, 4B, 4C1, 4C2, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -1600,6 +1730,11 @@
           <t>197</t>
         </is>
       </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -1607,6 +1742,11 @@
           <t>198</t>
         </is>
       </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -1614,6 +1754,11 @@
           <t>199</t>
         </is>
       </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C1, 1C2, 2A, 2B, 2C, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -1621,11 +1766,21 @@
           <t>2</t>
         </is>
       </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
           <t>20</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 7 village workbooks (sivaramans-llin 2026-10-08T18:06:17Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Chennavaram_13.464802_80.149579.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Chennavaram_13.464802_80.149579.xlsx
@@ -1790,6 +1790,11 @@
           <t>200</t>
         </is>
       </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -1797,6 +1802,11 @@
           <t>201</t>
         </is>
       </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -1804,6 +1814,11 @@
           <t>202</t>
         </is>
       </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -1811,6 +1826,11 @@
           <t>203</t>
         </is>
       </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -1818,6 +1838,11 @@
           <t>204</t>
         </is>
       </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -1825,6 +1850,11 @@
           <t>205</t>
         </is>
       </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 1C, 2, 3A1, 3A2, 3A3, 3A4, 3A5, 3A6, 3B1A, 3B1B, 3B2, 4A, 4B, 4C, 4D1, 4D2, 4D3</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -1832,6 +1862,11 @@
           <t>206</t>
         </is>
       </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C, 3D, 3E, 3F</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -1839,6 +1874,11 @@
           <t>207</t>
         </is>
       </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 1C, 1D, 1E1, 1E2, 1E3, 1E4A, 1E4B, 1E5, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -1846,11 +1886,21 @@
           <t>208</t>
         </is>
       </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C1, 1C2, 1C3, 1C4, 1C5, 1C6A, 1C6B, 1C7A, 1C7B, 1D1, 1D2, 1E1, 1E2, 2</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
           <t>209</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 8 village workbooks (sivaramans-llin 2026-10-08T18:10:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Chennavaram_13.464802_80.149579.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Chennavaram_13.464802_80.149579.xlsx
@@ -1910,6 +1910,11 @@
           <t>21</t>
         </is>
       </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -1917,6 +1922,11 @@
           <t>210</t>
         </is>
       </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>1A1, 1A2A, 1A2B, 1B1, 1B2, 1B3, 1B4, 1B5, 1B6A, 1B6B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -1924,6 +1934,11 @@
           <t>211</t>
         </is>
       </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B1, 3B2, 3C, 3D, 3E, 3F, 3G, 3H, 3I</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -1931,6 +1946,11 @@
           <t>212</t>
         </is>
       </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -1938,6 +1958,11 @@
           <t>213</t>
         </is>
       </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -1945,6 +1970,11 @@
           <t>214</t>
         </is>
       </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -1952,6 +1982,11 @@
           <t>215</t>
         </is>
       </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -1959,6 +1994,11 @@
           <t>216</t>
         </is>
       </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -1966,6 +2006,11 @@
           <t>217</t>
         </is>
       </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>1, 1B1, 1B2, 1C, 2A, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -1973,6 +2018,11 @@
           <t>218</t>
         </is>
       </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C, 2D, 2E1, 2E2, 2F, 3A, 3B, 3C1, 3C2, 3D, 3E, 3F, 3G, 3H, 3I, 3J, 3K, 3L, 3M, 3N1, 3N2, 3N3, 3O, 3P1, 3P2, 3P3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -1980,6 +2030,11 @@
           <t>219</t>
         </is>
       </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>1A, 1B1A, 1B1B, 1B2, 2</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -1987,6 +2042,11 @@
           <t>22</t>
         </is>
       </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2A3, 2A4, 2B, 2C1, 2C2A1, 2C2A2, 2C2B</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -1994,6 +2054,11 @@
           <t>220</t>
         </is>
       </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1B3, 2A, 2B, 2C, 2D, 2E, 2F, 2G, 2H, 2I1, 2I2, 2J1, 2K, 2L, 2M, 2N, 2O, 2P, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -2001,6 +2066,11 @@
           <t>221</t>
         </is>
       </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>10, 11, 1A, 1B, 2A, 2B, 2C, 2D1, 2D2, 3A1, 3A2, 3B, 4A, 4B, 4C, 4D, 4E, 4F, 4G, 4H, 4I, 4J, 5, 6A, 6B1, 6B2, 6C, 6D1, 6D2A1, 6D2B, 6D2C, 6E1A, 6E1B, 6E1C, 6E1D, 6E2, 7A, 7B1A, 7B1B, 7B2A, 7B2B1, 7B2B2, 7B2B3, 8, 9A1A, 9A1B, 9A2, 9A3, 9A4, 9A5, 9A6, 9B, 9C, 9D</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -2008,6 +2078,11 @@
           <t>222</t>
         </is>
       </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2A1A1, 2A1A2A1A, 2A1A2B, 2A1A2C, 2A1A2D, 2A1A2E, 2A1B1, 2A1B2, 2A2A, 2A2B, 2B1, 2B2, 2B3, 3, 4, 5A1A1, 5A2, 5B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -2015,6 +2090,11 @@
           <t>223</t>
         </is>
       </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -2022,6 +2102,11 @@
           <t>23</t>
         </is>
       </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -2029,6 +2114,11 @@
           <t>24</t>
         </is>
       </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -2036,6 +2126,11 @@
           <t>25</t>
         </is>
       </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -2043,6 +2138,11 @@
           <t>26</t>
         </is>
       </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -2050,6 +2150,11 @@
           <t>27</t>
         </is>
       </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C, 2D1, 2D2, 2D3, 2D4, 3</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -2057,6 +2162,11 @@
           <t>28</t>
         </is>
       </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1A, 1B1B, 1B2, 1B3A, 1B3B, 1B4, 2</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -2064,6 +2174,11 @@
           <t>29</t>
         </is>
       </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -2071,6 +2186,11 @@
           <t>3</t>
         </is>
       </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -2078,6 +2198,11 @@
           <t>30</t>
         </is>
       </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -2085,6 +2210,11 @@
           <t>31</t>
         </is>
       </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 4C</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -2092,6 +2222,11 @@
           <t>32</t>
         </is>
       </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B, 4, 5A1, 5A2, 5B1, 5B2</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -2099,6 +2234,11 @@
           <t>33</t>
         </is>
       </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -2106,6 +2246,11 @@
           <t>34</t>
         </is>
       </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C1, 1C2, 1D, 1E1, 1E2, 2A, 2B, 3A, 3B, 4A, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -2113,6 +2258,11 @@
           <t>35</t>
         </is>
       </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -2120,6 +2270,11 @@
           <t>36</t>
         </is>
       </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -2127,6 +2282,11 @@
           <t>37</t>
         </is>
       </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7A, 7B, 7C, 8A, 8B</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -2134,6 +2294,11 @@
           <t>38</t>
         </is>
       </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5A, 5B, 5C, 6A, 6B, 7A, 7B, 8</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -2141,6 +2306,11 @@
           <t>39</t>
         </is>
       </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -2148,6 +2318,11 @@
           <t>4</t>
         </is>
       </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -2155,6 +2330,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -2162,11 +2342,21 @@
           <t>41</t>
         </is>
       </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
           <t>42</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 9 village workbooks (sivaramans-llin 2026-10-08T18:20:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Chennavaram_13.464802_80.149579.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Chennavaram_13.464802_80.149579.xlsx
@@ -2366,6 +2366,11 @@
           <t>43</t>
         </is>
       </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B, 2A, 2B, 2C, 2D, 2E</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -2373,6 +2378,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B1, 3B2</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -2380,6 +2390,11 @@
           <t>45</t>
         </is>
       </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -2387,6 +2402,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -2394,6 +2414,11 @@
           <t>47</t>
         </is>
       </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1A4, 1A5A, 1A5B, 1B1, 1B2, 1B3, 1B4, 1B5, 1B6, 1B7, 1B8, 1C1, 1C2, 1C3, 1C4, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -2401,6 +2426,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -2408,6 +2438,11 @@
           <t>49</t>
         </is>
       </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C, 3D, 3E, 3F, 3G, 3H, 3I, 4A, 4B, 4C, 4D, 5A, 5B1, 5B2, 5B3</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -2415,6 +2450,11 @@
           <t>5</t>
         </is>
       </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -2422,6 +2462,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -2429,6 +2474,11 @@
           <t>51</t>
         </is>
       </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -2436,6 +2486,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -2443,6 +2498,11 @@
           <t>53</t>
         </is>
       </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -2450,6 +2510,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -2457,6 +2522,11 @@
           <t>55</t>
         </is>
       </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -2464,6 +2534,11 @@
           <t>56</t>
         </is>
       </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -2471,6 +2546,11 @@
           <t>57</t>
         </is>
       </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -2478,6 +2558,11 @@
           <t>58</t>
         </is>
       </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -2485,6 +2570,11 @@
           <t>59</t>
         </is>
       </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>1A1A, 1B, 1C, 1D, 1E, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -2492,6 +2582,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -2499,6 +2594,11 @@
           <t>60</t>
         </is>
       </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -2506,6 +2606,11 @@
           <t>61</t>
         </is>
       </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C, 3D, 3E</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -2513,6 +2618,11 @@
           <t>62</t>
         </is>
       </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -2520,6 +2630,11 @@
           <t>63</t>
         </is>
       </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -2527,6 +2642,11 @@
           <t>64</t>
         </is>
       </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -2534,6 +2654,11 @@
           <t>65</t>
         </is>
       </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -2541,6 +2666,11 @@
           <t>66</t>
         </is>
       </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>1, 2, 3A1, 3A2, 3B, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -2548,6 +2678,11 @@
           <t>67</t>
         </is>
       </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -2555,6 +2690,11 @@
           <t>68</t>
         </is>
       </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -2562,6 +2702,11 @@
           <t>69</t>
         </is>
       </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -2569,6 +2714,11 @@
           <t>7</t>
         </is>
       </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -2576,6 +2726,11 @@
           <t>70</t>
         </is>
       </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -2583,6 +2738,11 @@
           <t>71</t>
         </is>
       </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -2590,6 +2750,11 @@
           <t>72</t>
         </is>
       </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 2E, 2F, 3, 4A, 4B, 4C</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -2597,6 +2762,11 @@
           <t>73</t>
         </is>
       </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -2604,6 +2774,11 @@
           <t>74</t>
         </is>
       </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -2611,6 +2786,11 @@
           <t>75</t>
         </is>
       </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>1A1, 1A10A, 1A10B, 1A11, 1A12, 1A13, 1A2, 1A3, 1A4, 1A5, 1A6, 1A7, 1A8, 1A9, 1B, 2A, 2B1, 2B2, 2B3, 2B4, 2B5, 2B6, 2B7, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -2618,6 +2798,11 @@
           <t>76</t>
         </is>
       </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -2625,6 +2810,11 @@
           <t>77</t>
         </is>
       </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B1, 2B2, 3A, 3B, 3C, 3D, 3E</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -2632,6 +2822,11 @@
           <t>78</t>
         </is>
       </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>1A1, 1A2A, 1A2B, 1B, 2, 3A, 3B, 4A, 4B, 5A, 5B1, 5B2</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -2639,6 +2834,11 @@
           <t>79</t>
         </is>
       </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -2646,6 +2846,11 @@
           <t>8</t>
         </is>
       </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3A, 3B, 4, 5, 6, 7A, 7B, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -2653,6 +2858,11 @@
           <t>80</t>
         </is>
       </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -2660,6 +2870,11 @@
           <t>81</t>
         </is>
       </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 2E</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -2667,6 +2882,11 @@
           <t>82</t>
         </is>
       </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 2, 3A1, 3A2, 3B, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -2674,6 +2894,11 @@
           <t>83</t>
         </is>
       </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -2681,6 +2906,11 @@
           <t>84</t>
         </is>
       </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A1C, 1A2, 1A3, 1B, 2A, 2B, 2C, 2D, 2E, 2F, 2G, 2H, 2J, 2K1, 3A, 3B, 3C</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -2688,6 +2918,11 @@
           <t>85</t>
         </is>
       </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>1, 2, 3A1, 3A2, 3B, 4A, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -2695,6 +2930,11 @@
           <t>86</t>
         </is>
       </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -2702,6 +2942,11 @@
           <t>87</t>
         </is>
       </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -2709,6 +2954,11 @@
           <t>88</t>
         </is>
       </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -2716,6 +2966,11 @@
           <t>89</t>
         </is>
       </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -2723,6 +2978,11 @@
           <t>9</t>
         </is>
       </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1C, 2A, 2B, 3, 4, 5, 6A, 6B</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -2730,6 +2990,11 @@
           <t>90</t>
         </is>
       </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2A, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -2737,6 +3002,11 @@
           <t>91</t>
         </is>
       </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D1, 2D2, 3A, 3B, 3C, 3D</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -2744,6 +3014,11 @@
           <t>92</t>
         </is>
       </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -2751,6 +3026,11 @@
           <t>93</t>
         </is>
       </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -2758,6 +3038,11 @@
           <t>94</t>
         </is>
       </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -2765,6 +3050,11 @@
           <t>95</t>
         </is>
       </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -2772,6 +3062,11 @@
           <t>96</t>
         </is>
       </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -2779,6 +3074,11 @@
           <t>97</t>
         </is>
       </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -2786,11 +3086,21 @@
           <t>98</t>
         </is>
       </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C1, 2C2, 2D, 2E, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
           <t>99</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>10, 1A, 1B, 2A, 2B, 3, 4, 5A, 5B, 5C, 5D, 5E, 6, 7A, 7B, 8, 9</t>
         </is>
       </c>
     </row>

</xml_diff>